<commit_message>
fix X button and added proctors department
</commit_message>
<xml_diff>
--- a/data/import/dummy_proctors.xlsx
+++ b/data/import/dummy_proctors.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Proctors" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,25 +426,20 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C156"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>DEPARTMENT</t>
         </is>
@@ -670,7 +677,11 @@
           <t>christopher.villarete@edu.ph</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -751,7 +762,11 @@
           <t>daniel.macaspac@edu.ph</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -764,7 +779,11 @@
           <t>daniel.mateo@edu.ph</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -777,7 +796,11 @@
           <t>daniel.sison@edu.ph</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -807,7 +830,11 @@
           <t>daniel.vargas@edu.ph</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -820,7 +847,11 @@
           <t>daniel.villaganas@edu.ph</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -833,7 +864,11 @@
           <t>david.gongora@edu.ph</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -846,7 +881,11 @@
           <t>david.guerrero@edu.ph</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -876,7 +915,11 @@
           <t>david.payusan@edu.ph</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -906,7 +949,11 @@
           <t>david.villarete@edu.ph</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -936,7 +983,11 @@
           <t>elizabeth.delapena@edu.ph</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -949,7 +1000,11 @@
           <t>elizabeth.flores@edu.ph</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -962,7 +1017,11 @@
           <t>elizabeth.garcia@edu.ph</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1179,7 +1238,11 @@
           <t>karen.sison@edu.ph</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1226,7 +1289,11 @@
           <t>karen.villaganas@edu.ph</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1256,7 +1323,11 @@
           <t>kertney.cali@edu.ph</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1286,7 +1357,11 @@
           <t>kertney.onlagada@edu.ph</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1316,7 +1391,11 @@
           <t>kertney.santos@edu.ph</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1363,7 +1442,11 @@
           <t>linda.bundang@edu.ph</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1376,7 +1459,11 @@
           <t>linda.cali@edu.ph</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1457,7 +1544,11 @@
           <t>lisa.flores@edu.ph</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1572,7 +1663,11 @@
           <t>margaret.cadiente@edu.ph</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1602,7 +1697,11 @@
           <t>margaret.macaspac@edu.ph</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1615,7 +1714,11 @@
           <t>margaret.payusan@edu.ph</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1628,7 +1731,11 @@
           <t>margaret.villarete@edu.ph</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1726,7 +1833,11 @@
           <t>matthew.pasco@edu.ph</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1773,7 +1884,11 @@
           <t>michael.buenafrancisca@edu.ph</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1786,7 +1901,11 @@
           <t>michael.bundang@edu.ph</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1799,7 +1918,11 @@
           <t>michael.giray@edu.ph</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1829,7 +1952,11 @@
           <t>michael.maraya@edu.ph</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1842,7 +1969,11 @@
           <t>michael.mateo@edu.ph</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1855,7 +1986,11 @@
           <t>michael.nuque@edu.ph</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1868,7 +2003,11 @@
           <t>michael.sanjuan@edu.ph</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2102,7 +2241,11 @@
           <t>patricia.garcia@edu.ph</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2115,7 +2258,11 @@
           <t>patricia.gascon@edu.ph</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2145,7 +2292,11 @@
           <t>patricia.santos@edu.ph</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2226,7 +2377,11 @@
           <t>richard.garcia@edu.ph</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2307,7 +2462,11 @@
           <t>robert.macaspac@edu.ph</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2320,7 +2479,11 @@
           <t>robert.sison@edu.ph</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2333,7 +2496,11 @@
           <t>robert.villaganas@edu.ph</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2363,7 +2530,11 @@
           <t>sarah.cali@edu.ph</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2393,7 +2564,11 @@
           <t>sarah.mariano@edu.ph</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2474,7 +2649,11 @@
           <t>susan.cali@edu.ph</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2504,7 +2683,11 @@
           <t>susan.guerrero@edu.ph</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2517,7 +2700,11 @@
           <t>susan.mariano@edu.ph</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2564,7 +2751,11 @@
           <t>susan.pasco@edu.ph</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2645,7 +2836,11 @@
           <t>susan.villarete@edu.ph</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2675,7 +2870,11 @@
           <t>thomas.delapena@edu.ph</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2705,7 +2904,11 @@
           <t>thomas.salem@edu.ph</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr"/>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2735,7 +2938,11 @@
           <t>thomas.sison@edu.ph</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2782,7 +2989,11 @@
           <t>william.buenafrancisca@edu.ph</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2795,7 +3006,11 @@
           <t>william.flores@edu.ph</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2859,7 +3074,11 @@
           <t>william.villarete@edu.ph</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SHS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>